<commit_message>
Adjust evals for expected behavior
</commit_message>
<xml_diff>
--- a/skills/skill-test/example/ccdi-federation-copilot-mvp.xlsx
+++ b/skills/skill-test/example/ccdi-federation-copilot-mvp.xlsx
@@ -965,7 +965,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>States eye_color is not a supported field/PV; does not invent.</t>
+          <t>Pass if the response states that eye_color is not a harmonized subject field and/or is not defined in bundled subject PV metadata. It may present metadata.unharmonized.eye_color=blue (GET or curl) as the unharmonized API filter shape, including case-sensitivity or node-variation caveats. Fail only if it claims eye_color/blue is a validated harmonized controlled subject field or PV, or presents a bare harmonized filter like ?eye_color=blue as supported.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>For this intentionally vague prompt, a general or bounded CCDI Federation metadata answer is acceptable. Pass if the response: (1) states assumptions about pediatric context and how "cancer" is interpreted; (2) documents the API endpoint/params used or what would be queried; (3) includes caveats or limitations (e.g. no reliable age filter, no single generic cancer PV, node errors). Live bounded fetch is acceptable when the user says "show me". Follow-up questions are optional. Fail only if the response invents facts with confidence, omits major ambiguities without any caveat, or presents incorrect API behavior as certain.</t>
+          <t>For this intentionally vague prompt, either path is acceptable. Pass if: (A) the response identifies material ambiguity (e.g. pediatric age cutoff and/or cancer/cohort scope) and asks a focused clarifying question before fetching or asserting a definitive cohort; or (B) it provides a bounded metadata answer with working assumptions (pediatric + cancer interpretation), documents endpoint/params or the planned query, and includes relevant caveats/limitations. Live bounded fetch is acceptable when the user says "show me". Fail only if the response invents facts with confidence, treats the vague prompt as unambiguous with no caveat or clarification, or presents incorrect API behavior as certain.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>F, M, U, UNDIFFERENTIATED from bundled PV metadata.</t>
+          <t>Pass if the response lists all four bundled subject sex codes: F, M, U, and UNDIFFERENTIATED. Labels from bundled PV metadata (Female, Male, Unknown, Intersex) and caDSR CDE 6343385 v1.00 / bundled-PV provenance are acceptable. Ignore unrelated skill version or release-check notes. Fail only if a required code is missing, a non-bundled sex code is presented as allowed, or the answer contradicts the bundled subject PV metadata.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">

</xml_diff>